<commit_message>
📊 Actualizar RECLUTAMIENTO_ASESORES_ACTIVOS_SEMANAL.xlsx — 13-04-2026, 4:06:33 p. m.
</commit_message>
<xml_diff>
--- a/datos/RECLUTAMIENTO_ASESORES_ACTIVOS_SEMANAL.xlsx
+++ b/datos/RECLUTAMIENTO_ASESORES_ACTIVOS_SEMANAL.xlsx
@@ -8,13 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{89D56589-BC6D-4D98-8361-94944E97E742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{89D56589-BC6D-4D98-8361-94944E97E742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF1C7E89-D7A1-44B5-BD32-1921B25A2CB3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{185AB9BF-E552-4A26-B63B-689E222494DE}"/>
   </bookViews>
   <sheets>
     <sheet name="ACTIVOS" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'[1]abril-26'!$AK$1:$AL$125</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1991,12 +1997,1038 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="WALTER"/>
+      <sheetName val="CAMILO"/>
+      <sheetName val="Hoja1"/>
+      <sheetName val="abril-26"/>
+      <sheetName val="Listas"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3">
+        <row r="1">
+          <cell r="AK1" t="str">
+            <v>RUT</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="AK2" t="str">
+            <v>26517777-8</v>
+          </cell>
+          <cell r="AL2" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="AK3" t="str">
+            <v>21300348-8</v>
+          </cell>
+          <cell r="AL3" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="AK4" t="str">
+            <v>9479309-2</v>
+          </cell>
+          <cell r="AL4" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="AK5" t="str">
+            <v>16647721-2</v>
+          </cell>
+          <cell r="AL5" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="AK6" t="str">
+            <v>28731281-4</v>
+          </cell>
+          <cell r="AL6" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="AK7" t="str">
+            <v>19658366-1</v>
+          </cell>
+          <cell r="AL7" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="AK8" t="str">
+            <v>15151770-6</v>
+          </cell>
+          <cell r="AL8" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="AK9" t="str">
+            <v>27207379-1</v>
+          </cell>
+          <cell r="AL9" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="AK10" t="str">
+            <v>12272359-3</v>
+          </cell>
+          <cell r="AL10" t="e">
+            <v>#N/A</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="AK11" t="str">
+            <v>25855121-4</v>
+          </cell>
+          <cell r="AL11" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="AK12" t="str">
+            <v>15083647-6</v>
+          </cell>
+          <cell r="AL12" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="AK13" t="str">
+            <v>13786667-6</v>
+          </cell>
+          <cell r="AL13" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="AK14" t="str">
+            <v>12856176-5</v>
+          </cell>
+          <cell r="AL14" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="AK15" t="str">
+            <v>13438762-9</v>
+          </cell>
+          <cell r="AL15" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="AK16" t="str">
+            <v>17231805-3</v>
+          </cell>
+          <cell r="AL16" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="AK17" t="str">
+            <v>11197545-0</v>
+          </cell>
+          <cell r="AL17" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="AK18" t="str">
+            <v>13831497-9</v>
+          </cell>
+          <cell r="AL18" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="AK19" t="str">
+            <v>15510038-9</v>
+          </cell>
+          <cell r="AL19" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="AK20" t="str">
+            <v>19912697-0</v>
+          </cell>
+          <cell r="AL20" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="AK21" t="str">
+            <v>19183023-7</v>
+          </cell>
+          <cell r="AL21" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="AK22" t="str">
+            <v>19241498-9</v>
+          </cell>
+          <cell r="AL22" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="AK23" t="str">
+            <v>19618782-0</v>
+          </cell>
+          <cell r="AL23" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="AK24" t="str">
+            <v>14413170-3</v>
+          </cell>
+          <cell r="AL24" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="AK25" t="str">
+            <v>19548383-3</v>
+          </cell>
+          <cell r="AL25" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="AK26" t="str">
+            <v>18152581-9</v>
+          </cell>
+          <cell r="AL26" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="AK27" t="str">
+            <v>14750432-2</v>
+          </cell>
+          <cell r="AL27" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="AK28" t="str">
+            <v>15082784-1</v>
+          </cell>
+          <cell r="AL28" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="AK29" t="str">
+            <v>16230736-3</v>
+          </cell>
+          <cell r="AL29" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="AK30" t="str">
+            <v>15632219-9</v>
+          </cell>
+          <cell r="AL30" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="AK31" t="str">
+            <v>8004652-9</v>
+          </cell>
+          <cell r="AL31" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="AK32" t="str">
+            <v>13063224-6</v>
+          </cell>
+          <cell r="AL32" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="AK33" t="str">
+            <v>20706766-0</v>
+          </cell>
+          <cell r="AL33" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="34">
+          <cell r="AK34" t="str">
+            <v>26494648-4</v>
+          </cell>
+          <cell r="AL34" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="35">
+          <cell r="AK35" t="str">
+            <v>14153741-5</v>
+          </cell>
+          <cell r="AL35" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="36">
+          <cell r="AK36" t="str">
+            <v>26154821-6</v>
+          </cell>
+          <cell r="AL36" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="37">
+          <cell r="AK37" t="str">
+            <v>18661183-7</v>
+          </cell>
+          <cell r="AL37" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="38">
+          <cell r="AK38" t="str">
+            <v>13896930-4</v>
+          </cell>
+          <cell r="AL38" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="39">
+          <cell r="AK39" t="str">
+            <v>19080830-0</v>
+          </cell>
+          <cell r="AL39" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="40">
+          <cell r="AK40" t="str">
+            <v>15728090-2</v>
+          </cell>
+          <cell r="AL40" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="41">
+          <cell r="AK41" t="str">
+            <v>22702441-0</v>
+          </cell>
+          <cell r="AL41" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="42">
+          <cell r="AK42" t="str">
+            <v>12460674-8</v>
+          </cell>
+          <cell r="AL42" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="43">
+          <cell r="AK43" t="str">
+            <v>22451053-5</v>
+          </cell>
+          <cell r="AL43" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="44">
+          <cell r="AK44" t="str">
+            <v>16362980-1</v>
+          </cell>
+          <cell r="AL44" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="45">
+          <cell r="AK45" t="str">
+            <v>27261703-1</v>
+          </cell>
+          <cell r="AL45" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="46">
+          <cell r="AK46" t="str">
+            <v>13878158-5</v>
+          </cell>
+          <cell r="AL46" t="e">
+            <v>#N/A</v>
+          </cell>
+        </row>
+        <row r="47">
+          <cell r="AK47" t="str">
+            <v>19238090-1</v>
+          </cell>
+          <cell r="AL47" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="48">
+          <cell r="AK48" t="str">
+            <v>28905767-6</v>
+          </cell>
+          <cell r="AL48" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="49">
+          <cell r="AK49" t="str">
+            <v>26744348-3</v>
+          </cell>
+          <cell r="AL49" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="50">
+          <cell r="AK50" t="str">
+            <v>9189905-1</v>
+          </cell>
+          <cell r="AL50" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="51">
+          <cell r="AK51" t="str">
+            <v>25728060-8</v>
+          </cell>
+          <cell r="AL51" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="52">
+          <cell r="AK52" t="str">
+            <v>16115129-7</v>
+          </cell>
+          <cell r="AL52" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="53">
+          <cell r="AK53" t="str">
+            <v>20476289-9</v>
+          </cell>
+          <cell r="AL53" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="54">
+          <cell r="AK54" t="str">
+            <v>28079891-6</v>
+          </cell>
+          <cell r="AL54" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="55">
+          <cell r="AK55" t="str">
+            <v>24416009-3</v>
+          </cell>
+          <cell r="AL55" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="56">
+          <cell r="AK56" t="str">
+            <v>17060336-2</v>
+          </cell>
+          <cell r="AL56" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="57">
+          <cell r="AK57" t="str">
+            <v>21541249-0</v>
+          </cell>
+          <cell r="AL57" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="58">
+          <cell r="AK58" t="str">
+            <v>10770302-0</v>
+          </cell>
+          <cell r="AL58" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="59">
+          <cell r="AK59" t="str">
+            <v>21662126-3</v>
+          </cell>
+          <cell r="AL59" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="60">
+          <cell r="AK60" t="str">
+            <v>19499412-5</v>
+          </cell>
+          <cell r="AL60" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="61">
+          <cell r="AK61" t="str">
+            <v>21725309-8</v>
+          </cell>
+          <cell r="AL61" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="62">
+          <cell r="AK62" t="str">
+            <v>19064968-7</v>
+          </cell>
+          <cell r="AL62" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="63">
+          <cell r="AK63" t="str">
+            <v>18599859-2</v>
+          </cell>
+          <cell r="AL63" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="64">
+          <cell r="AK64" t="str">
+            <v>6875810-6</v>
+          </cell>
+          <cell r="AL64" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="65">
+          <cell r="AK65" t="str">
+            <v>18704172-4</v>
+          </cell>
+          <cell r="AL65" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="66">
+          <cell r="AK66" t="str">
+            <v>9617670-8</v>
+          </cell>
+          <cell r="AL66" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="67">
+          <cell r="AK67" t="str">
+            <v>15557591-3</v>
+          </cell>
+          <cell r="AL67" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="68">
+          <cell r="AK68" t="str">
+            <v>26639684-8</v>
+          </cell>
+          <cell r="AL68" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="69">
+          <cell r="AK69" t="str">
+            <v>12021587-6</v>
+          </cell>
+          <cell r="AL69" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="70">
+          <cell r="AK70" t="str">
+            <v>10984092-0</v>
+          </cell>
+          <cell r="AL70" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="71">
+          <cell r="AK71" t="str">
+            <v>17313898-9</v>
+          </cell>
+          <cell r="AL71" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="72">
+          <cell r="AK72" t="str">
+            <v>6477736-K</v>
+          </cell>
+          <cell r="AL72" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="73">
+          <cell r="AK73" t="str">
+            <v>26062269-0</v>
+          </cell>
+          <cell r="AL73" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="74">
+          <cell r="AK74" t="str">
+            <v>8517880-6</v>
+          </cell>
+          <cell r="AL74" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="75">
+          <cell r="AK75" t="str">
+            <v>15898487-3</v>
+          </cell>
+          <cell r="AL75" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="76">
+          <cell r="AK76" t="str">
+            <v>13289205-9</v>
+          </cell>
+          <cell r="AL76" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="77">
+          <cell r="AK77" t="str">
+            <v>20944439-9</v>
+          </cell>
+          <cell r="AL77" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="78">
+          <cell r="AK78" t="str">
+            <v>17091997-1</v>
+          </cell>
+          <cell r="AL78" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="79">
+          <cell r="AK79">
+            <v>258265874</v>
+          </cell>
+          <cell r="AL79" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="80">
+          <cell r="AK80" t="str">
+            <v>21502132-7</v>
+          </cell>
+          <cell r="AL80" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="81">
+          <cell r="AK81" t="str">
+            <v>16453949-0</v>
+          </cell>
+          <cell r="AL81" t="e">
+            <v>#N/A</v>
+          </cell>
+        </row>
+        <row r="82">
+          <cell r="AK82" t="str">
+            <v>19287852-7</v>
+          </cell>
+          <cell r="AL82" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="83">
+          <cell r="AK83" t="str">
+            <v>13696856-4</v>
+          </cell>
+          <cell r="AL83" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="84">
+          <cell r="AK84" t="str">
+            <v>10471701-2</v>
+          </cell>
+          <cell r="AL84" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="85">
+          <cell r="AK85" t="str">
+            <v>26282940-5</v>
+          </cell>
+          <cell r="AL85" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="86">
+          <cell r="AK86" t="str">
+            <v>19182462-8</v>
+          </cell>
+          <cell r="AL86" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="87">
+          <cell r="AK87" t="str">
+            <v>16421508-3</v>
+          </cell>
+          <cell r="AL87" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="88">
+          <cell r="AK88" t="str">
+            <v>26432326-6</v>
+          </cell>
+          <cell r="AL88" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="89">
+          <cell r="AK89" t="str">
+            <v>16021016-8</v>
+          </cell>
+          <cell r="AL89" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="90">
+          <cell r="AK90" t="str">
+            <v>20192333-6</v>
+          </cell>
+          <cell r="AL90" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="91">
+          <cell r="AK91" t="str">
+            <v>18467872-1</v>
+          </cell>
+          <cell r="AL91" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="92">
+          <cell r="AK92" t="str">
+            <v>21797287-6</v>
+          </cell>
+          <cell r="AL92" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="93">
+          <cell r="AK93" t="str">
+            <v>14582270-K</v>
+          </cell>
+          <cell r="AL93" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="94">
+          <cell r="AK94" t="str">
+            <v>26808914-4</v>
+          </cell>
+          <cell r="AL94" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="95">
+          <cell r="AK95" t="str">
+            <v>19471670-2</v>
+          </cell>
+          <cell r="AL95" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="96">
+          <cell r="AK96" t="str">
+            <v>20131637-5</v>
+          </cell>
+          <cell r="AL96" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="97">
+          <cell r="AK97" t="str">
+            <v>10207590-0</v>
+          </cell>
+          <cell r="AL97" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="98">
+          <cell r="AK98" t="str">
+            <v>19438826-8</v>
+          </cell>
+          <cell r="AL98" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="99">
+          <cell r="AK99" t="str">
+            <v>26180199-K</v>
+          </cell>
+          <cell r="AL99" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="100">
+          <cell r="AK100" t="str">
+            <v>26209853-2</v>
+          </cell>
+          <cell r="AL100" t="e">
+            <v>#N/A</v>
+          </cell>
+        </row>
+        <row r="101">
+          <cell r="AK101" t="str">
+            <v>20330542-7</v>
+          </cell>
+          <cell r="AL101" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="102">
+          <cell r="AK102" t="str">
+            <v>19615029-3</v>
+          </cell>
+          <cell r="AL102" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="103">
+          <cell r="AK103" t="str">
+            <v>16231137-9</v>
+          </cell>
+          <cell r="AL103" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="104">
+          <cell r="AK104" t="str">
+            <v>19721334-5</v>
+          </cell>
+          <cell r="AL104" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="105">
+          <cell r="AK105" t="str">
+            <v>17836080-9</v>
+          </cell>
+          <cell r="AL105" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="106">
+          <cell r="AK106" t="str">
+            <v>17675115-0</v>
+          </cell>
+          <cell r="AL106" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="107">
+          <cell r="AK107" t="str">
+            <v>16800740-K</v>
+          </cell>
+          <cell r="AL107" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="108">
+          <cell r="AK108" t="str">
+            <v>20183421-K</v>
+          </cell>
+          <cell r="AL108" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="109">
+          <cell r="AK109" t="str">
+            <v>18354796-8</v>
+          </cell>
+          <cell r="AL109" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="110">
+          <cell r="AK110" t="str">
+            <v>19739643-1</v>
+          </cell>
+          <cell r="AL110" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="111">
+          <cell r="AK111" t="str">
+            <v>16006609-1</v>
+          </cell>
+          <cell r="AL111" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="112">
+          <cell r="AK112" t="str">
+            <v>17304704-5</v>
+          </cell>
+          <cell r="AL112" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="113">
+          <cell r="AK113" t="str">
+            <v>12774636-2</v>
+          </cell>
+          <cell r="AL113" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="114">
+          <cell r="AK114" t="str">
+            <v>12830056-2</v>
+          </cell>
+          <cell r="AL114" t="e">
+            <v>#N/A</v>
+          </cell>
+        </row>
+        <row r="115">
+          <cell r="AK115" t="str">
+            <v>18189757-0</v>
+          </cell>
+          <cell r="AL115" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="116">
+          <cell r="AK116" t="str">
+            <v>18121387-6</v>
+          </cell>
+          <cell r="AL116" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="117">
+          <cell r="AK117" t="str">
+            <v>11642539-4</v>
+          </cell>
+          <cell r="AL117" t="e">
+            <v>#N/A</v>
+          </cell>
+        </row>
+        <row r="118">
+          <cell r="AK118" t="str">
+            <v>20277802-K</v>
+          </cell>
+          <cell r="AL118" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="119">
+          <cell r="AK119" t="str">
+            <v>27421822-3</v>
+          </cell>
+          <cell r="AL119" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="120">
+          <cell r="AK120" t="str">
+            <v>29122024-K</v>
+          </cell>
+          <cell r="AL120" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="121">
+          <cell r="AK121" t="str">
+            <v>18243548-1</v>
+          </cell>
+          <cell r="AL121" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="122">
+          <cell r="AK122" t="str">
+            <v>27109000-5</v>
+          </cell>
+          <cell r="AL122" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="123">
+          <cell r="AK123">
+            <v>184301512</v>
+          </cell>
+          <cell r="AL123" t="str">
+            <v>INACTIVO</v>
+          </cell>
+        </row>
+        <row r="124">
+          <cell r="AK124" t="str">
+            <v>20221783-4</v>
+          </cell>
+          <cell r="AL124" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+        <row r="125">
+          <cell r="AK125" t="str">
+            <v>27504210-2</v>
+          </cell>
+          <cell r="AL125" t="str">
+            <v>ACTIVO</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="4"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D3D9A7A3-2A7A-4756-A134-1A60675456D4}" name="Tabla2" displayName="Tabla2" ref="A1:AA125" totalsRowShown="0">
   <autoFilter ref="A1:AA125" xr:uid="{D3D9A7A3-2A7A-4756-A134-1A60675456D4}">
     <filterColumn colId="3">
       <filters>
-        <filter val="CAMILO MEDEL"/>
+        <filter val="WALTER FERRO"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -2327,27 +3359,27 @@
     <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="47.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="36.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="40.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.44140625" customWidth="1"/>
+    <col min="8" max="8" width="21.88671875" customWidth="1"/>
+    <col min="9" max="9" width="10.77734375" customWidth="1"/>
+    <col min="10" max="10" width="26.21875" customWidth="1"/>
+    <col min="11" max="11" width="47.5546875" customWidth="1"/>
+    <col min="12" max="12" width="16.21875" customWidth="1"/>
+    <col min="13" max="13" width="36.77734375" customWidth="1"/>
+    <col min="14" max="14" width="11.33203125" customWidth="1"/>
+    <col min="15" max="15" width="24.88671875" customWidth="1"/>
+    <col min="16" max="16" width="16.33203125" customWidth="1"/>
+    <col min="17" max="17" width="16.77734375" customWidth="1"/>
+    <col min="18" max="18" width="40.109375" customWidth="1"/>
+    <col min="19" max="19" width="20.21875" customWidth="1"/>
+    <col min="20" max="20" width="10.77734375" customWidth="1"/>
+    <col min="21" max="21" width="15.33203125" customWidth="1"/>
+    <col min="22" max="22" width="13.88671875" customWidth="1"/>
+    <col min="23" max="23" width="12.21875" customWidth="1"/>
+    <col min="24" max="24" width="10.77734375" customWidth="1"/>
+    <col min="25" max="25" width="13.77734375" customWidth="1"/>
+    <col min="26" max="26" width="10.77734375" customWidth="1"/>
+    <col min="27" max="27" width="24.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
@@ -2492,7 +3524,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -2681,7 +3713,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -2743,7 +3775,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3177,7 +4209,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -3245,7 +4277,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -3404,7 +4436,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -4567,7 +5599,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>98</v>
       </c>
@@ -4635,7 +5667,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -4700,7 +5732,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -4765,7 +5797,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>18</v>
       </c>
@@ -4833,7 +5865,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -5208,7 +6240,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -5326,7 +6358,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -5456,7 +6488,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="51" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -5648,7 +6680,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -5710,7 +6742,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="55" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>13</v>
       </c>
@@ -5834,7 +6866,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -6011,7 +7043,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>13</v>
       </c>
@@ -6259,7 +7291,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -6616,7 +7648,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="70" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>18</v>
       </c>
@@ -6935,7 +7967,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>13</v>
       </c>
@@ -6994,7 +8026,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>13</v>
       </c>
@@ -7059,7 +8091,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="77" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>13</v>
       </c>
@@ -7277,7 +8309,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="81" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>18</v>
       </c>
@@ -7339,7 +8371,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="82" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -7720,7 +8752,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="88" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>13</v>
       </c>
@@ -7779,7 +8811,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>13</v>
       </c>
@@ -8053,7 +9085,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="94" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>18</v>
       </c>
@@ -8304,7 +9336,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="98" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>13</v>
       </c>
@@ -8366,7 +9398,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="99" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>13</v>
       </c>
@@ -8856,7 +9888,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="107" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>13</v>
       </c>
@@ -8921,7 +9953,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="108" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>13</v>
       </c>
@@ -8983,7 +10015,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="109" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>13</v>
       </c>
@@ -9201,7 +10233,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="113" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>98</v>
       </c>
@@ -9272,7 +10304,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="114" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>18</v>
       </c>
@@ -9340,7 +10372,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="115" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>13</v>
       </c>
@@ -9402,7 +10434,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="116" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>13</v>
       </c>
@@ -9585,7 +10617,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="119" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>13</v>
       </c>
@@ -9771,7 +10803,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="122" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>13</v>
       </c>
@@ -9839,7 +10871,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="123" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>13</v>
       </c>

</xml_diff>